<commit_message>
Remove Elastic Feeds. Start and fix Pytest with several upgrades in RSTools like off-line entities
</commit_message>
<xml_diff>
--- a/formshare/tests/resources/forms/form06.xlsx
+++ b/formshare/tests/resources/forms/form06.xlsx
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -180,7 +180,7 @@
     <t xml:space="preserve">Just a test</t>
   </si>
   <si>
-    <t xml:space="preserve">Justtest</t>
+    <t xml:space="preserve">Justtest_6</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
@@ -271,28 +271,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -308,152 +312,258 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="13.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.71484375" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="35.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="29.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="28.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="23.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="21.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1020" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="29.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="28.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="23.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1020" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -469,172 +579,172 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="13.71484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.71484375" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1023" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1023" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="0" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="0" t="s">
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="4"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="4"/>
+      <c r="D8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="0" t="s">
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="B13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="0" t="s">
+      <c r="B14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -650,44 +760,44 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="9.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.60546875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>